<commit_message>
Send pending batch 2026-10-07-1715
</commit_message>
<xml_diff>
--- a/inbox/pending.xlsx
+++ b/inbox/pending.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="90">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -281,6 +281,9 @@
   </si>
   <si>
     <t>claremont@haven.org.za</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -651,6 +654,9 @@
       <c r="D2" t="s">
         <v>51</v>
       </c>
+      <c r="G2" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
@@ -665,6 +671,9 @@
       <c r="D3" t="s">
         <v>52</v>
       </c>
+      <c r="G3" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
@@ -679,6 +688,9 @@
       <c r="D4" t="s">
         <v>53</v>
       </c>
+      <c r="G4" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -693,6 +705,9 @@
       <c r="D5" t="s">
         <v>54</v>
       </c>
+      <c r="G5" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -707,6 +722,9 @@
       <c r="D6" t="s">
         <v>55</v>
       </c>
+      <c r="G6" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -721,6 +739,9 @@
       <c r="D7" t="s">
         <v>56</v>
       </c>
+      <c r="G7" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -735,6 +756,9 @@
       <c r="D8" t="s">
         <v>57</v>
       </c>
+      <c r="G8" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -749,6 +773,9 @@
       <c r="D9" t="s">
         <v>58</v>
       </c>
+      <c r="G9" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -763,6 +790,9 @@
       <c r="D10" t="s">
         <v>59</v>
       </c>
+      <c r="G10" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -777,6 +807,9 @@
       <c r="D11" t="s">
         <v>60</v>
       </c>
+      <c r="G11" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
@@ -791,6 +824,9 @@
       <c r="D12" t="s">
         <v>61</v>
       </c>
+      <c r="G12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
@@ -805,6 +841,9 @@
       <c r="D13" t="s">
         <v>62</v>
       </c>
+      <c r="G13" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
@@ -819,6 +858,9 @@
       <c r="D14" t="s">
         <v>63</v>
       </c>
+      <c r="G14" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
@@ -833,6 +875,9 @@
       <c r="D15" t="s">
         <v>64</v>
       </c>
+      <c r="G15" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
@@ -847,8 +892,11 @@
       <c r="D16" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="G16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -861,8 +909,11 @@
       <c r="D17" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="G17" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -875,8 +926,11 @@
       <c r="D18" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="G18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -889,8 +943,11 @@
       <c r="D19" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="G19" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -903,8 +960,11 @@
       <c r="D20" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="G20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -917,8 +977,11 @@
       <c r="D21" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="G21" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -931,8 +994,11 @@
       <c r="D22" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="G22" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -945,8 +1011,11 @@
       <c r="D23" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="G23" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -959,8 +1028,11 @@
       <c r="D24" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="G24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -973,8 +1045,11 @@
       <c r="D25" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="G25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -987,8 +1062,11 @@
       <c r="D26" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="G26" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -1001,8 +1079,11 @@
       <c r="D27" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="G27" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -1015,8 +1096,11 @@
       <c r="D28" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="G28" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -1029,8 +1113,11 @@
       <c r="D29" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="G29" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -1043,8 +1130,11 @@
       <c r="D30" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
+      <c r="G30" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -1057,8 +1147,11 @@
       <c r="D31" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="G31" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1071,8 +1164,11 @@
       <c r="D32" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="G32" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -1085,8 +1181,11 @@
       <c r="D33" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="G33" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -1099,8 +1198,11 @@
       <c r="D34" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="G34" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -1113,8 +1215,11 @@
       <c r="D35" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="G35" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -1127,8 +1232,11 @@
       <c r="D36" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="G36" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -1141,8 +1249,11 @@
       <c r="D37" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="G37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -1155,8 +1266,11 @@
       <c r="D38" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="G38" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>44</v>
       </c>
@@ -1168,6 +1282,9 @@
       </c>
       <c r="D39" t="s">
         <v>88</v>
+      </c>
+      <c r="G39" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>